<commit_message>
Businessplan: Szenarien- und Sensitivitätswerte im Excel, Textbereinigung, Doku Miete 8,50 €/m²
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014T3huvdFuELAS4McTZt8zb
</commit_message>
<xml_diff>
--- a/gym-planner/businessplan/Finanzplan_No1.xlsx
+++ b/gym-planner/businessplan/Finanzplan_No1.xlsx
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="699" uniqueCount="509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="744" uniqueCount="549">
   <si>
     <t xml:space="preserve">Finanzplanung No.1 Fitness &amp; HYROX Studio (Arbeitstitel)</t>
   </si>
@@ -1737,6 +1737,126 @@
   </si>
   <si>
     <t xml:space="preserve">optimistisch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neuzugänge-Faktor / Kündigungsquote / Beitragsniveau</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,70 / 2,8 % / 0,95</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,00 / 2,2 % / 1,00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,20 / 1,8 % / 1,03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mitglieder Ende Jahr 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mitglieder Ende Jahr 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mitglieder Ende Jahr 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umsatz Jahr 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umsatz Jahr 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Umsatz Jahr 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITDA Jahr 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITDA Jahr 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITDA Jahr 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jahresergebnis Jahr 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jahresergebnis Jahr 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jahresergebnis Jahr 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jahresergebnis Jahr 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DSCR Jahr 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DSCR Jahr 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Niedrigster Kassenbestand (Monat)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-1.201.214 € (Monat 60)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">102.470 € (Monat 17)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">278.223 € (Monat -5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservebedarf 24 Monate inkl. Puffer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erster Monat EBITDA ≥ 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Erster Monat Cashflow nach Kapitaldienst ≥ 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n. e.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Break-even Mitglieder (Vollkosten M36)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sensitivitäten (Basis-Szenario, jeweils eine Annahme verändert; Werte)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ergebnis Jahr 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reservebedarf 24 Mon.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neuzugänge −20 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Neuzugänge −30 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kündigungsquote 3,0 %/Monat (statt 2,2 %)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Beitragsniveau −10 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kaltmiete 10,00 €/m² (statt 8,50 €)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zinsen +1,5 Prozentpunkte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Personalkosten +10 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Energie/Wasser 5,50 €/m² (statt 4,00 €)</t>
   </si>
 </sst>
 </file>
@@ -2841,12 +2961,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="B1:E4"/>
+  <dimension ref="B1:H38"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="3" style="0" width="18"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2871,6 +2991,535 @@
       </c>
       <c r="E4" s="30" t="s">
         <v>508</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B5" s="2" t="s">
+        <v>509</v>
+      </c>
+      <c r="C5" s="41" t="s">
+        <v>510</v>
+      </c>
+      <c r="D5" s="41" t="s">
+        <v>511</v>
+      </c>
+      <c r="E5" s="41" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="2" t="s">
+        <v>513</v>
+      </c>
+      <c r="C6" s="25" t="n">
+        <v>959</v>
+      </c>
+      <c r="D6" s="25" t="n">
+        <v>1429</v>
+      </c>
+      <c r="E6" s="25" t="n">
+        <v>1763</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B7" s="2" t="s">
+        <v>514</v>
+      </c>
+      <c r="C7" s="25" t="n">
+        <v>1332</v>
+      </c>
+      <c r="D7" s="25" t="n">
+        <v>2053</v>
+      </c>
+      <c r="E7" s="25" t="n">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="2" t="s">
+        <v>515</v>
+      </c>
+      <c r="C8" s="25" t="n">
+        <v>1525</v>
+      </c>
+      <c r="D8" s="25" t="n">
+        <v>2200</v>
+      </c>
+      <c r="E8" s="25" t="n">
+        <v>2200</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B9" s="2" t="s">
+        <v>516</v>
+      </c>
+      <c r="C9" s="25" t="n">
+        <v>408704</v>
+      </c>
+      <c r="D9" s="25" t="n">
+        <v>622361</v>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>776846</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="2" t="s">
+        <v>517</v>
+      </c>
+      <c r="C10" s="25" t="n">
+        <v>698004</v>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>1101585</v>
+      </c>
+      <c r="E10" s="25" t="n">
+        <v>1346015</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="2" t="s">
+        <v>518</v>
+      </c>
+      <c r="C11" s="25" t="n">
+        <v>871770</v>
+      </c>
+      <c r="D11" s="25" t="n">
+        <v>1375456</v>
+      </c>
+      <c r="E11" s="25" t="n">
+        <v>1431686</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="2" t="s">
+        <v>519</v>
+      </c>
+      <c r="C12" s="25" t="n">
+        <v>-584413</v>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>-376292</v>
+      </c>
+      <c r="E12" s="25" t="n">
+        <v>-225713</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="2" t="s">
+        <v>520</v>
+      </c>
+      <c r="C13" s="25" t="n">
+        <v>-226272</v>
+      </c>
+      <c r="D13" s="25" t="n">
+        <v>166583</v>
+      </c>
+      <c r="E13" s="25" t="n">
+        <v>404793</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="2" t="s">
+        <v>521</v>
+      </c>
+      <c r="C14" s="25" t="n">
+        <v>-71358</v>
+      </c>
+      <c r="D14" s="25" t="n">
+        <v>419028</v>
+      </c>
+      <c r="E14" s="25" t="n">
+        <v>474414</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="2" t="s">
+        <v>522</v>
+      </c>
+      <c r="C15" s="25" t="n">
+        <v>-990373</v>
+      </c>
+      <c r="D15" s="25" t="n">
+        <v>-782252</v>
+      </c>
+      <c r="E15" s="25" t="n">
+        <v>-631674</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="2" t="s">
+        <v>523</v>
+      </c>
+      <c r="C16" s="25" t="n">
+        <v>-585853</v>
+      </c>
+      <c r="D16" s="25" t="n">
+        <v>-192997</v>
+      </c>
+      <c r="E16" s="25" t="n">
+        <v>45212</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="2" t="s">
+        <v>524</v>
+      </c>
+      <c r="C17" s="25" t="n">
+        <v>-429741</v>
+      </c>
+      <c r="D17" s="25" t="n">
+        <v>60645</v>
+      </c>
+      <c r="E17" s="25" t="n">
+        <v>116031</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="2" t="s">
+        <v>525</v>
+      </c>
+      <c r="C18" s="25" t="n">
+        <v>-281845</v>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>104206</v>
+      </c>
+      <c r="E18" s="25" t="n">
+        <v>144428</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B19" s="2" t="s">
+        <v>526</v>
+      </c>
+      <c r="C19" s="23" t="n">
+        <v>-0.35</v>
+      </c>
+      <c r="D19" s="23" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="E19" s="23" t="n">
+        <v>2.31</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B20" s="2" t="s">
+        <v>527</v>
+      </c>
+      <c r="C20" s="23" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="D20" s="23" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="E20" s="23" t="n">
+        <v>1.8</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B21" s="2" t="s">
+        <v>528</v>
+      </c>
+      <c r="C21" s="41" t="s">
+        <v>529</v>
+      </c>
+      <c r="D21" s="41" t="s">
+        <v>530</v>
+      </c>
+      <c r="E21" s="41" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="2" t="s">
+        <v>532</v>
+      </c>
+      <c r="C22" s="25" t="n">
+        <v>1352019</v>
+      </c>
+      <c r="D22" s="25" t="n">
+        <v>708838</v>
+      </c>
+      <c r="E22" s="25" t="n">
+        <v>496997</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="2" t="s">
+        <v>533</v>
+      </c>
+      <c r="C23" s="36" t="n">
+        <v>41</v>
+      </c>
+      <c r="D23" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="E23" s="36" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="2" t="s">
+        <v>534</v>
+      </c>
+      <c r="C24" s="36" t="s">
+        <v>535</v>
+      </c>
+      <c r="D24" s="36" t="n">
+        <v>19</v>
+      </c>
+      <c r="E24" s="36" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="2" t="s">
+        <v>536</v>
+      </c>
+      <c r="C25" s="25" t="n">
+        <v>2095</v>
+      </c>
+      <c r="D25" s="25" t="n">
+        <v>2006</v>
+      </c>
+      <c r="E25" s="25" t="n">
+        <v>1957</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B28" s="4" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="30" t="s">
+        <v>538</v>
+      </c>
+      <c r="C29" s="30" t="s">
+        <v>521</v>
+      </c>
+      <c r="D29" s="30" t="s">
+        <v>539</v>
+      </c>
+      <c r="E29" s="30" t="s">
+        <v>526</v>
+      </c>
+      <c r="F29" s="30" t="s">
+        <v>527</v>
+      </c>
+      <c r="G29" s="30" t="s">
+        <v>540</v>
+      </c>
+      <c r="H29" s="30" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="41" t="s">
+        <v>507</v>
+      </c>
+      <c r="C30" s="25" t="n">
+        <v>419028</v>
+      </c>
+      <c r="D30" s="25" t="n">
+        <v>60645</v>
+      </c>
+      <c r="E30" s="23" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="F30" s="23" t="n">
+        <v>1.65</v>
+      </c>
+      <c r="G30" s="25" t="n">
+        <v>708838</v>
+      </c>
+      <c r="H30" s="25" t="n">
+        <v>2053</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="41" t="s">
+        <v>541</v>
+      </c>
+      <c r="C31" s="25" t="n">
+        <v>186865</v>
+      </c>
+      <c r="D31" s="25" t="n">
+        <v>-171518</v>
+      </c>
+      <c r="E31" s="23" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="F31" s="23" t="n">
+        <v>1.26</v>
+      </c>
+      <c r="G31" s="25" t="n">
+        <v>1046452</v>
+      </c>
+      <c r="H31" s="25" t="n">
+        <v>1642</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B32" s="41" t="s">
+        <v>542</v>
+      </c>
+      <c r="C32" s="25" t="n">
+        <v>48716</v>
+      </c>
+      <c r="D32" s="25" t="n">
+        <v>-309667</v>
+      </c>
+      <c r="E32" s="23" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="F32" s="23" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G32" s="25" t="n">
+        <v>1239229</v>
+      </c>
+      <c r="H32" s="25" t="n">
+        <v>1437</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B33" s="41" t="s">
+        <v>543</v>
+      </c>
+      <c r="C33" s="25" t="n">
+        <v>307409</v>
+      </c>
+      <c r="D33" s="25" t="n">
+        <v>-50974</v>
+      </c>
+      <c r="E33" s="23" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F33" s="23" t="n">
+        <v>1.58</v>
+      </c>
+      <c r="G33" s="25" t="n">
+        <v>779379</v>
+      </c>
+      <c r="H33" s="25" t="n">
+        <v>1856</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B34" s="41" t="s">
+        <v>544</v>
+      </c>
+      <c r="C34" s="25" t="n">
+        <v>307998</v>
+      </c>
+      <c r="D34" s="25" t="n">
+        <v>-50385</v>
+      </c>
+      <c r="E34" s="23" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F34" s="23" t="n">
+        <v>1.23</v>
+      </c>
+      <c r="G34" s="25" t="n">
+        <v>823229</v>
+      </c>
+      <c r="H34" s="25" t="n">
+        <v>2053</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B35" s="41" t="s">
+        <v>545</v>
+      </c>
+      <c r="C35" s="25" t="n">
+        <v>382034</v>
+      </c>
+      <c r="D35" s="25" t="n">
+        <v>23083</v>
+      </c>
+      <c r="E35" s="23" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="F35" s="23" t="n">
+        <v>1.51</v>
+      </c>
+      <c r="G35" s="25" t="n">
+        <v>779488</v>
+      </c>
+      <c r="H35" s="25" t="n">
+        <v>2053</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B36" s="41" t="s">
+        <v>546</v>
+      </c>
+      <c r="C36" s="25" t="n">
+        <v>419028</v>
+      </c>
+      <c r="D36" s="25" t="n">
+        <v>23881</v>
+      </c>
+      <c r="E36" s="23" t="n">
+        <v>1.73</v>
+      </c>
+      <c r="F36" s="23" t="n">
+        <v>1.46</v>
+      </c>
+      <c r="G36" s="25" t="n">
+        <v>786173</v>
+      </c>
+      <c r="H36" s="25" t="n">
+        <v>2053</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B37" s="41" t="s">
+        <v>547</v>
+      </c>
+      <c r="C37" s="25" t="n">
+        <v>378467</v>
+      </c>
+      <c r="D37" s="25" t="n">
+        <v>20084</v>
+      </c>
+      <c r="E37" s="23" t="n">
+        <v>1.85</v>
+      </c>
+      <c r="F37" s="23" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G37" s="25" t="n">
+        <v>775480</v>
+      </c>
+      <c r="H37" s="25" t="n">
+        <v>2053</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="41" t="s">
+        <v>548</v>
+      </c>
+      <c r="C38" s="25" t="n">
+        <v>383471</v>
+      </c>
+      <c r="D38" s="25" t="n">
+        <v>24520</v>
+      </c>
+      <c r="E38" s="23" t="n">
+        <v>1.86</v>
+      </c>
+      <c r="F38" s="23" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="G38" s="25" t="n">
+        <v>772195</v>
+      </c>
+      <c r="H38" s="25" t="n">
+        <v>2053</v>
       </c>
     </row>
   </sheetData>

</xml_diff>